<commit_message>
Updates in Cancer Journey Date Evolution (conceptual)
</commit_message>
<xml_diff>
--- a/_sources/LogicalModelExample_v1.xlsx
+++ b/_sources/LogicalModelExample_v1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hl7europe-my.sharepoint.com/personal/roberta_hl7europe_org/Documents/Roberta/IDEA4RC/Cancer Model/LogicalModel/Esempi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{ED9382E8-2342-4AE0-AA39-3164F895D6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4FC69E83-2811-44BE-ABE9-7C5202981F0F}"/>
+  <xr:revisionPtr revIDLastSave="43" documentId="8_{ED9382E8-2342-4AE0-AA39-3164F895D6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB4339A7-18F0-4913-A8EE-D926D3B57F38}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DIAGNOSIS + FIRST TREATMENT" sheetId="1" r:id="rId1"/>
@@ -283,12 +283,6 @@
     <t>EvidenceReference</t>
   </si>
   <si>
-    <t>Imaging/44</t>
-  </si>
-  <si>
-    <t>Surgery/55</t>
-  </si>
-  <si>
     <t>Radiotherapy</t>
   </si>
   <si>
@@ -307,6 +301,12 @@
     <t>CodeSystem: SNOMED CT
 Code: 367336001
 DisplayName: Chemotherapy (procedure)</t>
+  </si>
+  <si>
+    <t>Imaging/1</t>
+  </si>
+  <si>
+    <t>Surgery/1</t>
   </si>
 </sst>
 </file>
@@ -765,7 +765,7 @@
       </c>
       <c r="Q1" s="22"/>
       <c r="S1" s="22" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="T1" s="22"/>
     </row>
@@ -780,37 +780,37 @@
         <v>0</v>
       </c>
       <c r="E2" s="2">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="H2" s="2">
-        <v>44</v>
+        <v>1</v>
       </c>
       <c r="J2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="K2" s="2">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="M2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="N2" s="2">
-        <v>55</v>
+        <v>1</v>
       </c>
       <c r="P2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="Q2" s="2">
-        <v>34</v>
+        <v>2</v>
       </c>
       <c r="S2" s="15" t="s">
         <v>0</v>
       </c>
       <c r="T2" s="2">
-        <v>15</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="135" x14ac:dyDescent="0.25">
@@ -836,25 +836,25 @@
         <v>58</v>
       </c>
       <c r="K3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="M3" s="10" t="s">
         <v>60</v>
       </c>
       <c r="N3" s="2">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="P3" s="10" t="s">
         <v>58</v>
       </c>
       <c r="Q3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="S3" s="2" t="s">
         <v>60</v>
       </c>
       <c r="T3" s="2">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="105" x14ac:dyDescent="0.25">
@@ -887,7 +887,7 @@
         <v>58</v>
       </c>
       <c r="N4" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>17</v>
@@ -899,7 +899,7 @@
         <v>58</v>
       </c>
       <c r="T4" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="75" x14ac:dyDescent="0.25">
@@ -996,7 +996,7 @@
         <v>70</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="M7" s="18" t="s">
         <v>26</v>
@@ -1008,7 +1008,7 @@
         <v>70</v>
       </c>
       <c r="Q7" s="2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="S7" s="2" t="s">
         <v>49</v>
@@ -1059,10 +1059,10 @@
         <v>43221</v>
       </c>
       <c r="S10" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11" spans="1:20" x14ac:dyDescent="0.25">
@@ -1140,19 +1140,19 @@
         <v>58</v>
       </c>
       <c r="B3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>58</v>
       </c>
       <c r="E3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>60</v>
       </c>
       <c r="H3" s="1">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -1309,13 +1309,13 @@
         <v>58</v>
       </c>
       <c r="B3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>60</v>
       </c>
       <c r="E3" s="1">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1453,13 +1453,13 @@
         <v>58</v>
       </c>
       <c r="B3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>60</v>
       </c>
       <c r="E3" s="1">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1597,13 +1597,13 @@
         <v>58</v>
       </c>
       <c r="B3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>60</v>
       </c>
       <c r="E3" s="1">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1729,7 +1729,7 @@
         <v>60</v>
       </c>
       <c r="B3" s="2">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1737,7 +1737,7 @@
         <v>58</v>
       </c>
       <c r="B4" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1761,7 +1761,7 @@
         <v>19</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1782,7 +1782,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>16</v>
@@ -1790,10 +1790,10 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1858,19 +1858,19 @@
         <v>58</v>
       </c>
       <c r="B3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>58</v>
       </c>
       <c r="E3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>60</v>
       </c>
       <c r="H3" s="1">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -2027,13 +2027,13 @@
         <v>58</v>
       </c>
       <c r="B3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>60</v>
       </c>
       <c r="E3" s="1">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2159,7 +2159,7 @@
         <v>60</v>
       </c>
       <c r="B3" s="1">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>